<commit_message>
Fix inspection tab: Add success message in modal and fix data table refresh
- Add message containers to both add and edit inspection modals
- Implement showMessage() and clearMessage() functions for modal feedback
- Update form submission handlers to show success message in modal before closing
- Fix dayjs undefined error by replacing with native JavaScript date methods
- Add comprehensive debugging and error handling for data table refresh
- Add test refresh button for debugging purposes
- Ensure data table refreshes properly after inspection operations
- Follow same pattern as site visit tab for consistent user experience
</commit_message>
<xml_diff>
--- a/resources/templates/unit-upload-template.xlsx
+++ b/resources/templates/unit-upload-template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="46">
   <si>
     <t>Unit Code</t>
   </si>
@@ -47,10 +47,28 @@
     <t>Miscellaneous Info</t>
   </si>
   <si>
-    <t>A101</t>
-  </si>
-  <si>
-    <t>Apartment 101</t>
+    <t>Address Line 1</t>
+  </si>
+  <si>
+    <t>Address Line 2</t>
+  </si>
+  <si>
+    <t>Address Line 3</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>County/State</t>
+  </si>
+  <si>
+    <t>Zip/EirCode</t>
+  </si>
+  <si>
+    <t>UNIT001</t>
+  </si>
+  <si>
+    <t>Apartment 1A</t>
   </si>
   <si>
     <t>John Doe</t>
@@ -59,22 +77,25 @@
     <t>Mr.</t>
   </si>
   <si>
-    <t>john.doe@example.com</t>
+    <t>john.doe@email.com</t>
   </si>
   <si>
     <t>Yes</t>
   </si>
   <si>
+    <t>0987654321</t>
+  </si>
+  <si>
     <t>ABC Properties</t>
   </si>
   <si>
-    <t>Sample information for unit A101</t>
-  </si>
-  <si>
-    <t>A102</t>
-  </si>
-  <si>
-    <t>Apartment 102</t>
+    <t>Resident lives in the unit</t>
+  </si>
+  <si>
+    <t>UNIT002</t>
+  </si>
+  <si>
+    <t>Office 2B</t>
   </si>
   <si>
     <t>Jane Smith</t>
@@ -83,70 +104,55 @@
     <t>Ms.</t>
   </si>
   <si>
-    <t>jane.smith@example.com</t>
+    <t>jane.smith@email.com</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>XYZ Properties</t>
-  </si>
-  <si>
-    <t>Sample information for unit A102</t>
-  </si>
-  <si>
-    <t>B201</t>
-  </si>
-  <si>
-    <t>Apartment 201</t>
-  </si>
-  <si>
-    <t>Mike Johnson</t>
-  </si>
-  <si>
-    <t>mike.johnson@example.com</t>
+    <t>XYZ Management</t>
+  </si>
+  <si>
+    <t>Non-resident unit</t>
+  </si>
+  <si>
+    <t>123 Business Street</t>
+  </si>
+  <si>
+    <t>Suite 2B</t>
+  </si>
+  <si>
+    <t>Dublin 2</t>
+  </si>
+  <si>
+    <t>Ireland</t>
+  </si>
+  <si>
+    <t>Dublin</t>
+  </si>
+  <si>
+    <t>D02 XY12</t>
+  </si>
+  <si>
+    <t>UNIT003</t>
+  </si>
+  <si>
+    <t>Apartment 3C</t>
+  </si>
+  <si>
+    <t>Bob Johnson</t>
+  </si>
+  <si>
+    <t>bob.johnson@email.com</t>
   </si>
   <si>
     <t>DEF Properties</t>
   </si>
   <si>
-    <t>Sample information for unit B201</t>
-  </si>
-  <si>
-    <t>B202</t>
-  </si>
-  <si>
-    <t>Apartment 202</t>
-  </si>
-  <si>
-    <t>Sarah Wilson</t>
-  </si>
-  <si>
-    <t>sarah.wilson@example.com</t>
-  </si>
-  <si>
-    <t>GHI Properties</t>
-  </si>
-  <si>
-    <t>Sample information for unit B202</t>
-  </si>
-  <si>
-    <t>C301</t>
-  </si>
-  <si>
-    <t>Apartment 301</t>
-  </si>
-  <si>
-    <t>David Brown</t>
-  </si>
-  <si>
-    <t>david.brown@example.com</t>
-  </si>
-  <si>
-    <t>JKL Properties</t>
-  </si>
-  <si>
-    <t>Sample information for unit C301</t>
+    <t>Another resident unit</t>
+  </si>
+  <si>
+    <t>NOTE: Address fields are only saved to database when Resident = "No"</t>
   </si>
 </sst>
 </file>
@@ -154,7 +160,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -173,6 +179,15 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF0066CC"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -183,32 +198,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2E8F0"/>
+        <fgColor rgb="FFE0E0E0"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -217,8 +217,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -518,22 +520,28 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="29.421" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="10.569" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="38.848" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="15" customWidth="true" style="0"/>
+    <col min="2" max="2" width="20" customWidth="true" style="0"/>
+    <col min="3" max="3" width="20" customWidth="true" style="0"/>
+    <col min="4" max="4" width="12" customWidth="true" style="0"/>
+    <col min="5" max="5" width="25" customWidth="true" style="0"/>
+    <col min="6" max="6" width="10" customWidth="true" style="0"/>
+    <col min="7" max="7" width="15" customWidth="true" style="0"/>
+    <col min="8" max="8" width="15" customWidth="true" style="0"/>
+    <col min="9" max="9" width="20" customWidth="true" style="0"/>
+    <col min="10" max="10" width="30" customWidth="true" style="0"/>
+    <col min="11" max="11" width="25" customWidth="true" style="0"/>
+    <col min="12" max="12" width="25" customWidth="true" style="0"/>
+    <col min="13" max="13" width="25" customWidth="true" style="0"/>
+    <col min="14" max="14" width="15" customWidth="true" style="0"/>
+    <col min="15" max="15" width="15" customWidth="true" style="0"/>
+    <col min="16" max="16" width="15" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -564,165 +572,154 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:10">
-      <c r="A2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="2">
+    <row r="2" spans="1:16">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2">
         <v>1234567890</v>
       </c>
-      <c r="H2" s="2">
-        <v>1234567891</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="H2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
     </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:16">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3">
+        <v>1234567890</v>
+      </c>
+      <c r="I3" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M3" t="s">
+        <v>35</v>
+      </c>
+      <c r="N3" t="s">
+        <v>36</v>
+      </c>
+      <c r="O3" t="s">
+        <v>37</v>
+      </c>
+      <c r="P3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="E4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="2">
-        <v>1234567892</v>
-      </c>
-      <c r="H3" s="2">
-        <v>1234567893</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="G4">
+        <v>1122334455</v>
+      </c>
+      <c r="H4">
+        <v>5566778899</v>
+      </c>
+      <c r="I4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K4"/>
+      <c r="L4"/>
+      <c r="M4"/>
+      <c r="N4"/>
+      <c r="O4"/>
+      <c r="P4"/>
     </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="2">
-        <v>1234567894</v>
-      </c>
-      <c r="H4" s="2">
-        <v>1234567895</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" s="2">
-        <v>1234567896</v>
-      </c>
-      <c r="H5" s="2">
-        <v>1234567897</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:16">
       <c r="A6" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="2">
-        <v>1234567898</v>
-      </c>
-      <c r="H6" s="2">
-        <v>1234567899</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove country and state columns from unit upload Excel functionality
- Updated BlockUnitController to remove country/state processing
- Modified Excel template to have 14 columns instead of 16
- Removed Country and County/State columns from template
- Added Address Line 1, Address Line 2, Address Line 3, Zip/EirCode columns
- Updated sample data with proper address examples
- Modified CSV processing to handle new column structure
- Updated view to reflect new required columns list
- Regenerated unit-upload-template.xlsx with new structure
- Maintained address logic: only saved when Resident = 'No'
</commit_message>
<xml_diff>
--- a/resources/templates/unit-upload-template.xlsx
+++ b/resources/templates/unit-upload-template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56">
   <si>
     <t>Unit Code</t>
   </si>
@@ -56,19 +56,13 @@
     <t>Address Line 3</t>
   </si>
   <si>
-    <t>Country</t>
-  </si>
-  <si>
-    <t>County/State</t>
-  </si>
-  <si>
     <t>Zip/EirCode</t>
   </si>
   <si>
-    <t>UNIT001</t>
-  </si>
-  <si>
-    <t>Apartment 1A</t>
+    <t>A101</t>
+  </si>
+  <si>
+    <t>Apartment 101</t>
   </si>
   <si>
     <t>John Doe</t>
@@ -77,25 +71,22 @@
     <t>Mr.</t>
   </si>
   <si>
-    <t>john.doe@email.com</t>
+    <t>john.doe@example.com</t>
   </si>
   <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>0987654321</t>
-  </si>
-  <si>
     <t>ABC Properties</t>
   </si>
   <si>
-    <t>Resident lives in the unit</t>
-  </si>
-  <si>
-    <t>UNIT002</t>
-  </si>
-  <si>
-    <t>Office 2B</t>
+    <t>Sample information for unit A101</t>
+  </si>
+  <si>
+    <t>A102</t>
+  </si>
+  <si>
+    <t>Apartment 102</t>
   </si>
   <si>
     <t>Jane Smith</t>
@@ -104,55 +95,94 @@
     <t>Ms.</t>
   </si>
   <si>
-    <t>jane.smith@email.com</t>
+    <t>jane.smith@example.com</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>XYZ Management</t>
-  </si>
-  <si>
-    <t>Non-resident unit</t>
-  </si>
-  <si>
-    <t>123 Business Street</t>
-  </si>
-  <si>
-    <t>Suite 2B</t>
+    <t>XYZ Properties</t>
+  </si>
+  <si>
+    <t>Sample information for unit A102</t>
+  </si>
+  <si>
+    <t>123 Main Street</t>
+  </si>
+  <si>
+    <t>Apt 102</t>
   </si>
   <si>
     <t>Dublin 2</t>
   </si>
   <si>
-    <t>Ireland</t>
-  </si>
-  <si>
-    <t>Dublin</t>
-  </si>
-  <si>
     <t>D02 XY12</t>
   </si>
   <si>
-    <t>UNIT003</t>
-  </si>
-  <si>
-    <t>Apartment 3C</t>
-  </si>
-  <si>
-    <t>Bob Johnson</t>
-  </si>
-  <si>
-    <t>bob.johnson@email.com</t>
+    <t>B201</t>
+  </si>
+  <si>
+    <t>Apartment 201</t>
+  </si>
+  <si>
+    <t>Mike Johnson</t>
+  </si>
+  <si>
+    <t>mike.johnson@example.com</t>
   </si>
   <si>
     <t>DEF Properties</t>
   </si>
   <si>
-    <t>Another resident unit</t>
-  </si>
-  <si>
-    <t>NOTE: Address fields are only saved to database when Resident = "No"</t>
+    <t>Sample information for unit B201</t>
+  </si>
+  <si>
+    <t>B202</t>
+  </si>
+  <si>
+    <t>Apartment 202</t>
+  </si>
+  <si>
+    <t>Sarah Wilson</t>
+  </si>
+  <si>
+    <t>sarah.wilson@example.com</t>
+  </si>
+  <si>
+    <t>GHI Properties</t>
+  </si>
+  <si>
+    <t>Sample information for unit B202</t>
+  </si>
+  <si>
+    <t>456 Oak Avenue</t>
+  </si>
+  <si>
+    <t>Unit 202</t>
+  </si>
+  <si>
+    <t>Cork City</t>
+  </si>
+  <si>
+    <t>T12 AB34</t>
+  </si>
+  <si>
+    <t>C301</t>
+  </si>
+  <si>
+    <t>Apartment 301</t>
+  </si>
+  <si>
+    <t>David Brown</t>
+  </si>
+  <si>
+    <t>david.brown@example.com</t>
+  </si>
+  <si>
+    <t>JKL Properties</t>
+  </si>
+  <si>
+    <t>Sample information for unit C301</t>
   </si>
 </sst>
 </file>
@@ -160,7 +190,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -179,15 +209,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b val="1"/>
-      <i val="1"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="11"/>
-      <color rgb="FF0066CC"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -198,17 +219,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE0E0E0"/>
+        <fgColor rgb="FFE2E8F0"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -217,10 +253,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -520,28 +554,26 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="true" style="0"/>
-    <col min="2" max="2" width="20" customWidth="true" style="0"/>
-    <col min="3" max="3" width="20" customWidth="true" style="0"/>
-    <col min="4" max="4" width="12" customWidth="true" style="0"/>
-    <col min="5" max="5" width="25" customWidth="true" style="0"/>
-    <col min="6" max="6" width="10" customWidth="true" style="0"/>
-    <col min="7" max="7" width="15" customWidth="true" style="0"/>
-    <col min="8" max="8" width="15" customWidth="true" style="0"/>
-    <col min="9" max="9" width="20" customWidth="true" style="0"/>
-    <col min="10" max="10" width="30" customWidth="true" style="0"/>
-    <col min="11" max="11" width="25" customWidth="true" style="0"/>
-    <col min="12" max="12" width="25" customWidth="true" style="0"/>
-    <col min="13" max="13" width="25" customWidth="true" style="0"/>
-    <col min="14" max="14" width="15" customWidth="true" style="0"/>
-    <col min="15" max="15" width="15" customWidth="true" style="0"/>
-    <col min="16" max="16" width="15" customWidth="true" style="0"/>
+    <col min="1" max="1" width="11.711" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="29.421" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="10.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="9" max="9" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="38.848" bestFit="true" customWidth="true" style="0"/>
+    <col min="11" max="11" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="13" max="13" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="14" max="14" width="13.997" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -584,143 +616,202 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="C2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="2">
+        <v>1234567890</v>
+      </c>
+      <c r="H2" s="2">
+        <v>1234567891</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
     </row>
-    <row r="2" spans="1:16">
-      <c r="A2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="3" spans="1:14">
+      <c r="A3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="2">
+        <v>1234567892</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1234567893</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2">
-        <v>1234567890</v>
-      </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" t="s">
-        <v>24</v>
-      </c>
-      <c r="K2"/>
-      <c r="L2"/>
-      <c r="M2"/>
-      <c r="N2"/>
-      <c r="O2"/>
-      <c r="P2"/>
+      <c r="G4" s="2">
+        <v>1234567894</v>
+      </c>
+      <c r="H4" s="2">
+        <v>1234567895</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
     </row>
-    <row r="3" spans="1:16">
-      <c r="A3" t="s">
+    <row r="5" spans="1:14">
+      <c r="A5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3">
-        <v>1234567890</v>
-      </c>
-      <c r="I3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K3" t="s">
-        <v>33</v>
-      </c>
-      <c r="L3" t="s">
-        <v>34</v>
-      </c>
-      <c r="M3" t="s">
-        <v>35</v>
-      </c>
-      <c r="N3" t="s">
-        <v>36</v>
-      </c>
-      <c r="O3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P3" t="s">
-        <v>38</v>
+      <c r="G5" s="2">
+        <v>1234567896</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1234567897</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
-      <c r="A4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" t="s">
+    <row r="6" spans="1:14">
+      <c r="A6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4">
-        <v>1122334455</v>
-      </c>
-      <c r="H4">
-        <v>5566778899</v>
-      </c>
-      <c r="I4" t="s">
-        <v>43</v>
-      </c>
-      <c r="J4" t="s">
-        <v>44</v>
-      </c>
-      <c r="K4"/>
-      <c r="L4"/>
-      <c r="M4"/>
-      <c r="N4"/>
-      <c r="O4"/>
-      <c r="P4"/>
-    </row>
-    <row r="6" spans="1:16">
-      <c r="A6" s="2" t="s">
-        <v>45</v>
-      </c>
+      <c r="G6" s="2">
+        <v>1234567898</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1234567899</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>